<commit_message>
Rename second income project
</commit_message>
<xml_diff>
--- a/outputs/one_person_company_profit_sprint.xlsx
+++ b/outputs/one_person_company_profit_sprint.xlsx
@@ -151,7 +151,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t>一人公司利润体检冲刺 Dashboard - 目标：14 天收款 5000 元以上；默认 4 单 × 1299 元</t>
+          <t>十二周年#021：第二收入赚10万元 Dashboard - 目标：2026-10-03 前累计赚 100000 元</t>
         </is>
       </c>
     </row>
@@ -199,7 +199,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <v>5000</v>
+        <v>100000</v>
       </c>
       <c r="C4"/>
       <c r="D4" t="inlineStr">
@@ -402,7 +402,7 @@
         </is>
       </c>
       <c r="E11">
-        <f>IF(B5&gt;=5000,"OK","继续冲刺")</f>
+        <f>IF(B5&gt;=100000,"OK","继续冲刺")</f>
       </c>
       <c r="F11"/>
       <c r="G11"/>

</xml_diff>